<commit_message>
already fetched NPIs are skipped
</commit_message>
<xml_diff>
--- a/src/database/temp_outputs/combined_chunks_file.xlsx
+++ b/src/database/temp_outputs/combined_chunks_file.xlsx
@@ -1,84 +1,37 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Repositories\XpressCredentialling\src\database\temp_outputs\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{021AF42D-CA74-440F-B714-57CAFBF3306F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
-  <si>
-    <t>National Provider Identifier</t>
-  </si>
-  <si>
-    <t>Name</t>
-  </si>
-  <si>
-    <t>Email</t>
-  </si>
-  <si>
-    <t>1427085877</t>
-  </si>
-  <si>
-    <t>GRANT SEARLES</t>
-  </si>
-  <si>
-    <t>grantsearles@hotmail.com</t>
-  </si>
-  <si>
-    <t>1497844617</t>
-  </si>
-  <si>
-    <t>DAVID MILLER</t>
-  </si>
-  <si>
-    <t>David.Miller@UTSouthwestern.edu</t>
-  </si>
-  <si>
-    <t>1689630188</t>
-  </si>
-  <si>
-    <t>JOHN MATHEWS</t>
-  </si>
-  <si>
-    <t>michelle.mcclinton@bhsala.com</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <name val="Calibri"/>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -93,43 +46,93 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -417,52 +420,80 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>National Provider Identifier</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" t="s">
-        <v>5</v>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>1689630188</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>JOHN MATHEWS</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>michelle.mcclinton@bhsala.com</t>
+        </is>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" t="s">
-        <v>8</v>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>1497844617</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>DAVID MILLER</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>David.Miller@UTSouthwestern.edu</t>
+        </is>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" t="s">
-        <v>11</v>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>1427085877</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>GRANT SEARLES</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>grantsearles@hotmail.com</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
contains  non duplicated npi data
</commit_message>
<xml_diff>
--- a/src/database/temp_outputs/combined_chunks_file.xlsx
+++ b/src/database/temp_outputs/combined_chunks_file.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Repositories\XpressCredentialling\src\database\temp_outputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12747A20-6A26-4F81-8FBD-8D6C8CE20A0A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67AD7772-C939-4C53-BDB0-0719859F7F01}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="81">
   <si>
     <t>National Provider Identifier</t>
   </si>
@@ -31,40 +31,22 @@
     <t>Email</t>
   </si>
   <si>
-    <t>1427085877</t>
-  </si>
-  <si>
-    <t>GRANT SEARLES</t>
-  </si>
-  <si>
-    <t>grantsearles@hotmail.com</t>
-  </si>
-  <si>
-    <t>1497844617</t>
-  </si>
-  <si>
-    <t>DAVID MILLER</t>
-  </si>
-  <si>
-    <t>David.Miller@UTSouthwestern.edu</t>
-  </si>
-  <si>
-    <t>1689630188</t>
-  </si>
-  <si>
-    <t>JOHN MATHEWS</t>
-  </si>
-  <si>
-    <t>michelle.mcclinton@bhsala.com</t>
-  </si>
-  <si>
-    <t>1083678858</t>
-  </si>
-  <si>
-    <t>GREGORY DUNN</t>
-  </si>
-  <si>
-    <t>Gregory.Dunn@allina.com</t>
+    <t>1013914100</t>
+  </si>
+  <si>
+    <t>BEATRIX ARAIZA</t>
+  </si>
+  <si>
+    <t>trix155@hotmail.com</t>
+  </si>
+  <si>
+    <t>1578511861</t>
+  </si>
+  <si>
+    <t>MUHAMMAD HIZKIL</t>
+  </si>
+  <si>
+    <t>ayazhizkil@gmail.com</t>
   </si>
   <si>
     <t>1184693400</t>
@@ -74,6 +56,213 @@
   </si>
   <si>
     <t>JLAEM@bellsouth.net</t>
+  </si>
+  <si>
+    <t>1497794739</t>
+  </si>
+  <si>
+    <t>WAYNE BARRY</t>
+  </si>
+  <si>
+    <t>edpdoc@aol.com</t>
+  </si>
+  <si>
+    <t>1700862414</t>
+  </si>
+  <si>
+    <t>HECTOR LABRADA</t>
+  </si>
+  <si>
+    <t>liubilabra1@bellsouth.net</t>
+  </si>
+  <si>
+    <t>1467499285</t>
+  </si>
+  <si>
+    <t>JORGE SANTANDER</t>
+  </si>
+  <si>
+    <t>santander_MD@yahoo.com</t>
+  </si>
+  <si>
+    <t>1104875178</t>
+  </si>
+  <si>
+    <t>MARIANELA DE LA PORTILLA</t>
+  </si>
+  <si>
+    <t>nelyportilla@aol.com</t>
+  </si>
+  <si>
+    <t>1740373406</t>
+  </si>
+  <si>
+    <t>OFILIO ARGUELLO</t>
+  </si>
+  <si>
+    <t>darguell@bellsouth.net</t>
+  </si>
+  <si>
+    <t>1851528335</t>
+  </si>
+  <si>
+    <t>ERICH GERHARDT</t>
+  </si>
+  <si>
+    <t>Erich.gerhardt1@gmail.com</t>
+  </si>
+  <si>
+    <t>1093841728</t>
+  </si>
+  <si>
+    <t>DENNIS ROBISON</t>
+  </si>
+  <si>
+    <t>d.robison50@gmail.com</t>
+  </si>
+  <si>
+    <t>1437460854</t>
+  </si>
+  <si>
+    <t>JOHN HAGEDORN</t>
+  </si>
+  <si>
+    <t>Johnhagedorn@gmail.com</t>
+  </si>
+  <si>
+    <t>1790076826</t>
+  </si>
+  <si>
+    <t>ELISABETH JONES BROWN</t>
+  </si>
+  <si>
+    <t>raeraegomez@gmail.com</t>
+  </si>
+  <si>
+    <t>1790912228</t>
+  </si>
+  <si>
+    <t>TRAVIS HOLLOWAY</t>
+  </si>
+  <si>
+    <t>Travis.holloway2@hcahealthcare.com</t>
+  </si>
+  <si>
+    <t>1710274147</t>
+  </si>
+  <si>
+    <t>MICHAEL VAN HAL</t>
+  </si>
+  <si>
+    <t>vanvlietplasticsurgery@gmail.com</t>
+  </si>
+  <si>
+    <t>1003060211</t>
+  </si>
+  <si>
+    <t>VICHIN PURI</t>
+  </si>
+  <si>
+    <t>vichinpuri@mhd.com</t>
+  </si>
+  <si>
+    <t>1518910918</t>
+  </si>
+  <si>
+    <t>RAMON SASTRE</t>
+  </si>
+  <si>
+    <t>rafenuv@aol.com</t>
+  </si>
+  <si>
+    <t>1356436786</t>
+  </si>
+  <si>
+    <t>HUMBERTO FERNANDEZ-MIRO</t>
+  </si>
+  <si>
+    <t>mesmiro@gmail.com</t>
+  </si>
+  <si>
+    <t>1386646008</t>
+  </si>
+  <si>
+    <t>JAMES SCHUMACHER</t>
+  </si>
+  <si>
+    <t>april@sarasotaneurosurgery.com</t>
+  </si>
+  <si>
+    <t>1821046079</t>
+  </si>
+  <si>
+    <t>ALVARO OCAMPO</t>
+  </si>
+  <si>
+    <t>alomed@gmail.com</t>
+  </si>
+  <si>
+    <t>1669433801</t>
+  </si>
+  <si>
+    <t>TIMOTHY STERNBERG</t>
+  </si>
+  <si>
+    <t>timothy.l.sternberg.ctr@mail.mil</t>
+  </si>
+  <si>
+    <t>1073525747</t>
+  </si>
+  <si>
+    <t>PASQUALE DELL'API</t>
+  </si>
+  <si>
+    <t>dellapipx@yahoo.com</t>
+  </si>
+  <si>
+    <t>1689772881</t>
+  </si>
+  <si>
+    <t>MATTHEW DEMETREE</t>
+  </si>
+  <si>
+    <t>drmdemetree@bellsouth.net</t>
+  </si>
+  <si>
+    <t>1831170240</t>
+  </si>
+  <si>
+    <t>PEDRO TIRADO</t>
+  </si>
+  <si>
+    <t>pwtirado@me.com</t>
+  </si>
+  <si>
+    <t>1417945098</t>
+  </si>
+  <si>
+    <t>AVELINO CARIDE</t>
+  </si>
+  <si>
+    <t>gocanes83@att.net</t>
+  </si>
+  <si>
+    <t>1831175702</t>
+  </si>
+  <si>
+    <t>FRANCISCO ALVAREZ-GIL</t>
+  </si>
+  <si>
+    <t>falvarezgil@me.com</t>
+  </si>
+  <si>
+    <t>1346294337</t>
+  </si>
+  <si>
+    <t>EMMANUEL ROLDAN</t>
+  </si>
+  <si>
+    <t>eroldan65@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -138,7 +327,98 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="9">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -436,12 +716,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="19.6640625" customWidth="1"/>
-    <col min="2" max="2" width="23" customWidth="1"/>
-    <col min="3" max="3" width="30.88671875" customWidth="1"/>
+    <col min="1" max="1" width="17.44140625" customWidth="1"/>
+    <col min="2" max="2" width="24.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
@@ -510,7 +789,243 @@
         <v>17</v>
       </c>
     </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" t="s">
+        <v>22</v>
+      </c>
+      <c r="C8" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>24</v>
+      </c>
+      <c r="B9" t="s">
+        <v>25</v>
+      </c>
+      <c r="C9" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>27</v>
+      </c>
+      <c r="B10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C10" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>30</v>
+      </c>
+      <c r="B11" t="s">
+        <v>31</v>
+      </c>
+      <c r="C11" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>33</v>
+      </c>
+      <c r="B12" t="s">
+        <v>34</v>
+      </c>
+      <c r="C12" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>36</v>
+      </c>
+      <c r="B13" t="s">
+        <v>37</v>
+      </c>
+      <c r="C13" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>39</v>
+      </c>
+      <c r="B14" t="s">
+        <v>40</v>
+      </c>
+      <c r="C14" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>42</v>
+      </c>
+      <c r="B15" t="s">
+        <v>43</v>
+      </c>
+      <c r="C15" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>45</v>
+      </c>
+      <c r="B16" t="s">
+        <v>46</v>
+      </c>
+      <c r="C16" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>48</v>
+      </c>
+      <c r="B17" t="s">
+        <v>49</v>
+      </c>
+      <c r="C17" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>51</v>
+      </c>
+      <c r="B18" t="s">
+        <v>52</v>
+      </c>
+      <c r="C18" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>54</v>
+      </c>
+      <c r="B19" t="s">
+        <v>55</v>
+      </c>
+      <c r="C19" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>57</v>
+      </c>
+      <c r="B20" t="s">
+        <v>58</v>
+      </c>
+      <c r="C20" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>60</v>
+      </c>
+      <c r="B21" t="s">
+        <v>61</v>
+      </c>
+      <c r="C21" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>63</v>
+      </c>
+      <c r="B22" t="s">
+        <v>64</v>
+      </c>
+      <c r="C22" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>66</v>
+      </c>
+      <c r="B23" t="s">
+        <v>67</v>
+      </c>
+      <c r="C23" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>69</v>
+      </c>
+      <c r="B24" t="s">
+        <v>70</v>
+      </c>
+      <c r="C24" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>72</v>
+      </c>
+      <c r="B25" t="s">
+        <v>73</v>
+      </c>
+      <c r="C25" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>75</v>
+      </c>
+      <c r="B26" t="s">
+        <v>76</v>
+      </c>
+      <c r="C26" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>78</v>
+      </c>
+      <c r="B27" t="s">
+        <v>79</v>
+      </c>
+      <c r="C27" t="s">
+        <v>80</v>
+      </c>
+    </row>
   </sheetData>
+  <conditionalFormatting sqref="A1:XFD1048576">
+    <cfRule type="duplicateValues" dxfId="2" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>